<commit_message>
Create search page and add ingredients
Add search page so ingredients/foods can be added to a list
.
</commit_message>
<xml_diff>
--- a/sprints/sprint1/Sprint Backlog & Burnup Chart.xlsx
+++ b/sprints/sprint1/Sprint Backlog & Burnup Chart.xlsx
@@ -1257,10 +1257,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>

</xml_diff>

<commit_message>
Emi added hours to Sprint Backlog
</commit_message>
<xml_diff>
--- a/sprints/sprint1/Sprint Backlog & Burnup Chart.xlsx
+++ b/sprints/sprint1/Sprint Backlog & Burnup Chart.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a9e6f5ad0d3e00a8/Desktop/SE2Group5/Group5NutritionTracker/sprints/sprint1/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pikac\OneDrive\Desktop\Software Engineering\Group5NutritionTracker\sprints\sprint1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="21" documentId="13_ncr:1_{008A7FCF-852C-4EA3-9EB4-899CDDCDC630}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E045A2B3-F821-45FB-B04E-8131E9C1E5D3}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56295D35-69F0-4740-BAAC-E6F9E9CB1DC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="24220" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -432,10 +432,10 @@
                   <c:v>11.2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>23</c:v>
+                  <c:v>24.5</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>34.049999999999997</c:v>
+                  <c:v>39.549999999999997</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1521,15 +1521,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H32"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.81640625" customWidth="1"/>
-    <col min="2" max="2" width="67.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="41.7265625" style="7" customWidth="1"/>
-    <col min="4" max="4" width="14.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.77734375" customWidth="1"/>
+    <col min="2" max="2" width="67.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41.77734375" style="7" customWidth="1"/>
+    <col min="4" max="4" width="14.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="14" t="s">
         <v>8</v>
       </c>
@@ -1549,7 +1549,7 @@
       <c r="G1" s="11"/>
       <c r="H1" s="11"/>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="14"/>
       <c r="B2" s="12"/>
       <c r="C2" s="13"/>
@@ -1567,7 +1567,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>15</v>
       </c>
@@ -1576,12 +1576,20 @@
       </c>
       <c r="C3" s="8"/>
       <c r="D3" s="3"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4"/>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="E3" s="4">
+        <v>0</v>
+      </c>
+      <c r="F3" s="4">
+        <v>0</v>
+      </c>
+      <c r="G3" s="4">
+        <v>0</v>
+      </c>
+      <c r="H3" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>15</v>
       </c>
@@ -1590,12 +1598,20 @@
       </c>
       <c r="C4" s="8"/>
       <c r="D4" s="3"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="E4" s="4">
+        <v>0</v>
+      </c>
+      <c r="F4" s="4">
+        <v>0</v>
+      </c>
+      <c r="G4" s="4">
+        <v>1.5</v>
+      </c>
+      <c r="H4" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>16</v>
       </c>
@@ -1621,7 +1637,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>16</v>
       </c>
@@ -1647,7 +1663,7 @@
         <v>4.5</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>16</v>
       </c>
@@ -1673,7 +1689,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>16</v>
       </c>
@@ -1699,7 +1715,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>16</v>
       </c>
@@ -1725,7 +1741,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>16</v>
       </c>
@@ -1743,7 +1759,7 @@
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>18</v>
       </c>
@@ -1769,7 +1785,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>18</v>
       </c>
@@ -1795,7 +1811,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>17</v>
       </c>
@@ -1809,7 +1825,7 @@
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>17</v>
       </c>
@@ -1823,7 +1839,7 @@
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>17</v>
       </c>
@@ -1837,7 +1853,7 @@
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>18</v>
       </c>
@@ -1863,7 +1879,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>18</v>
       </c>
@@ -1889,7 +1905,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>18</v>
       </c>
@@ -1915,7 +1931,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>16</v>
       </c>
@@ -1933,7 +1949,7 @@
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
     </row>
-    <row r="20" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>16</v>
       </c>
@@ -1951,7 +1967,7 @@
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
     </row>
-    <row r="21" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>18</v>
       </c>
@@ -1977,7 +1993,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>17</v>
       </c>
@@ -1999,7 +2015,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>15</v>
       </c>
@@ -2008,12 +2024,20 @@
       </c>
       <c r="C23" s="8"/>
       <c r="D23" s="3"/>
-      <c r="E23" s="4"/>
-      <c r="F23" s="4"/>
-      <c r="G23" s="4"/>
-      <c r="H23" s="4"/>
-    </row>
-    <row r="24" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+      <c r="E23" s="4">
+        <v>0</v>
+      </c>
+      <c r="F23" s="4">
+        <v>0</v>
+      </c>
+      <c r="G23" s="4">
+        <v>0</v>
+      </c>
+      <c r="H23" s="4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>16</v>
       </c>
@@ -2031,7 +2055,7 @@
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
     </row>
-    <row r="25" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>16</v>
       </c>
@@ -2049,7 +2073,7 @@
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" s="2"/>
       <c r="B26" s="3"/>
       <c r="C26" s="8"/>
@@ -2059,7 +2083,7 @@
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" s="2"/>
       <c r="B27" s="3"/>
       <c r="C27" s="8"/>
@@ -2069,7 +2093,7 @@
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28" s="2"/>
       <c r="B28" s="3"/>
       <c r="C28" s="8"/>
@@ -2079,7 +2103,7 @@
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29" s="2"/>
       <c r="B29" s="3"/>
       <c r="C29" s="8"/>
@@ -2089,7 +2113,7 @@
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A30" s="2"/>
       <c r="B30" s="3"/>
       <c r="C30" s="8"/>
@@ -2099,7 +2123,7 @@
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A31" s="5"/>
       <c r="B31" s="5"/>
       <c r="C31" s="9" t="s">
@@ -2119,14 +2143,14 @@
       </c>
       <c r="G31" s="6">
         <f>SUM(G3:G30)+F31</f>
-        <v>23</v>
+        <v>24.5</v>
       </c>
       <c r="H31" s="6">
         <f>SUM(H3:H30)+G31</f>
-        <v>34.049999999999997</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
+        <v>39.549999999999997</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="E32">
         <f>D31</f>
         <v>42</v>

</xml_diff>